<commit_message>
résultats après reconfiguration des vType
</commit_message>
<xml_diff>
--- a/brt_config_files/current_config/data/graphiques/01_comparatif_global.xlsx
+++ b/brt_config_files/current_config/data/graphiques/01_comparatif_global.xlsx
@@ -445,13 +445,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>12.27</v>
+        <v>11.77</v>
       </c>
       <c r="B2" t="n">
-        <v>22.14</v>
+        <v>22.58</v>
       </c>
       <c r="C2" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -459,18 +459,18 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>24.616</v>
+        <v>23.51433333333334</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>6.29</v>
+        <v>5.05</v>
       </c>
       <c r="B3" t="n">
-        <v>43.15</v>
+        <v>50.51</v>
       </c>
       <c r="C3" t="n">
-        <v>99</v>
+        <v>319</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -478,18 +478,18 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>30.16066666666666</v>
+        <v>29.30833333333333</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>22.23</v>
+        <v>19.86</v>
       </c>
       <c r="B4" t="n">
-        <v>10.06</v>
+        <v>12.01</v>
       </c>
       <c r="C4" t="n">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>24.798</v>
+        <v>23.59633333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>